<commit_message>
Calibrate big-box categories in concise calculator
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ke8h4Zgp7WmQ6H3JyfNM4g
</commit_message>
<xml_diff>
--- a/output/Kalkulator_Anggaran_Interior_Toko_Ringkas.xlsx
+++ b/output/Kalkulator_Anggaran_Interior_Toko_Ringkas.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="100">
   <si>
     <t xml:space="preserve">PETUNJUK — Kalkulator Anggaran Interior Toko (versi ringkas)</t>
   </si>
@@ -111,6 +111,9 @@
     <t xml:space="preserve">• Sheet Parameter biasanya tidak perlu diubah.</t>
   </si>
   <si>
+    <t xml:space="preserve">• UPDATE: kategori perlengkapan rumah &amp; furnitur (big-box) sudah dikalibrasi dengan data agregat biaya fit-out toko baru.</t>
+  </si>
+  <si>
     <t xml:space="preserve">KALKULATOR ANGGARAN INTERIOR TOKO (versi ringkas)</t>
   </si>
   <si>
@@ -295,6 +298,9 @@
   </si>
   <si>
     <t xml:space="preserve">K = anggaran interior ÷ penjualan setahun. Biaya pasar = biaya interior per m² di MALL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KALIBRASI: dua kategori big-box memakai data agregat biaya fit-out toko baru. Kategori lain masih angka indikatif umum.</t>
   </si>
   <si>
     <t xml:space="preserve">TABEL 2 — Faktor lokasi (mengali biaya pasar)</t>
@@ -329,7 +335,7 @@
     <numFmt numFmtId="167" formatCode="0.0%;\-0.0%;\-"/>
     <numFmt numFmtId="168" formatCode="0.00\x"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -410,6 +416,14 @@
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -521,7 +535,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -655,6 +669,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -702,7 +720,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFC00000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -942,7 +960,7 @@
     <tabColor rgb="FF1F3864"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:C23"/>
+  <dimension ref="B1:C24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1079,6 +1097,11 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C23" s="5" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C24" s="5" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1118,23 +1141,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C3" s="12" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>7</v>
@@ -1142,7 +1165,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -1151,59 +1174,59 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>3000</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>2500000</v>
+        <v>1200000</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -1212,38 +1235,38 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C12" s="20" t="n">
         <f aca="false">C7*C8*12</f>
-        <v>90000000000</v>
+        <v>43200000000</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F14" s="21" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C15" s="22" t="n">
         <f aca="false">INDEX(Parameter!$B$6:$B$14,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
@@ -1251,19 +1274,19 @@
       </c>
       <c r="D15" s="23" t="n">
         <f aca="false">$C$12*C15</f>
-        <v>8100000000</v>
+        <v>3888000000</v>
       </c>
       <c r="E15" s="23" t="n">
         <f aca="false">IF($C$7&gt;0,D15/$C$7,0)</f>
-        <v>2700000</v>
+        <v>1296000</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C16" s="22" t="n">
         <f aca="false">AVERAGE(C15,C17)</f>
@@ -1271,19 +1294,19 @@
       </c>
       <c r="D16" s="23" t="n">
         <f aca="false">$C$12*C16</f>
-        <v>9900000000</v>
+        <v>4752000000</v>
       </c>
       <c r="E16" s="23" t="n">
         <f aca="false">IF($C$7&gt;0,D16/$C$7,0)</f>
-        <v>3300000</v>
+        <v>1584000</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C17" s="22" t="n">
         <f aca="false">INDEX(Parameter!$C$6:$C$14,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
@@ -1291,19 +1314,19 @@
       </c>
       <c r="D17" s="23" t="n">
         <f aca="false">$C$12*C17</f>
-        <v>11700000000</v>
+        <v>5616000000</v>
       </c>
       <c r="E17" s="23" t="n">
         <f aca="false">IF($C$7&gt;0,D17/$C$7,0)</f>
-        <v>3900000</v>
+        <v>1872000</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -1312,23 +1335,23 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C20" s="20" t="n">
-        <f aca="false">INDEX(Parameter!$D$6:$D$14,MATCH($C$6,Parameter!$A$6:$A$14,0))*INDEX(Parameter!$B$19:$B$20,MATCH($C$9,Parameter!$A$19:$A$20,0))</f>
-        <v>2000000</v>
+        <f aca="false">INDEX(Parameter!$D$6:$D$14,MATCH($C$6,Parameter!$A$6:$A$14,0))*INDEX(Parameter!$B$20:$B$21,MATCH($C$9,Parameter!$A$20:$A$21,0))</f>
+        <v>1000000</v>
       </c>
       <c r="D20" s="20" t="n">
-        <f aca="false">INDEX(Parameter!$E$6:$E$14,MATCH($C$6,Parameter!$A$6:$A$14,0))*INDEX(Parameter!$B$19:$B$20,MATCH($C$9,Parameter!$A$19:$A$20,0))</f>
-        <v>4000000</v>
+        <f aca="false">INDEX(Parameter!$E$6:$E$14,MATCH($C$6,Parameter!$A$6:$A$14,0))*INDEX(Parameter!$B$20:$B$21,MATCH($C$9,Parameter!$A$20:$A$21,0))</f>
+        <v>1600000</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C21" s="25" t="str">
         <f aca="false">IF(E16&gt;=D20,"LONGGAR — anggaran Standard di atas biaya pasar. Ada ruang untuk konsep lebih kuat.",IF(E16&gt;=C20,"SESUAI — anggaran Standard berada di kisaran biaya pasar. Desain kualitas menengah aman.","TIDAK CUKUP — anggaran di bawah biaya pasar. Sederhanakan desain atau cek ulang target penjualan dengan klien."))</f>
@@ -1340,7 +1363,7 @@
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -1349,123 +1372,123 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="21" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E24" s="21" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C25" s="22" t="n">
-        <f aca="false">INDEX(Parameter!$B$25:$B$33,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
+        <f aca="false">INDEX(Parameter!$B$26:$B$34,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
         <v>0.4</v>
       </c>
       <c r="D25" s="26" t="n">
         <f aca="false">$D$16*C25</f>
-        <v>3960000000</v>
+        <v>1900800000</v>
       </c>
       <c r="E25" s="20" t="n">
         <f aca="false">IF($C$7&gt;0,D25/$C$7,0)</f>
-        <v>1320000</v>
+        <v>633600</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C26" s="22" t="n">
-        <f aca="false">INDEX(Parameter!$C$25:$C$33,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
+        <f aca="false">INDEX(Parameter!$C$26:$C$34,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
         <v>0.17</v>
       </c>
       <c r="D26" s="26" t="n">
         <f aca="false">$D$16*C26</f>
-        <v>1683000000</v>
+        <v>807840000</v>
       </c>
       <c r="E26" s="20" t="n">
         <f aca="false">IF($C$7&gt;0,D26/$C$7,0)</f>
-        <v>561000</v>
+        <v>269280</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C27" s="22" t="n">
-        <f aca="false">INDEX(Parameter!$D$25:$D$33,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
+        <f aca="false">INDEX(Parameter!$D$26:$D$34,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
         <v>0.17</v>
       </c>
       <c r="D27" s="26" t="n">
         <f aca="false">$D$16*C27</f>
-        <v>1683000000</v>
+        <v>807840000</v>
       </c>
       <c r="E27" s="20" t="n">
         <f aca="false">IF($C$7&gt;0,D27/$C$7,0)</f>
-        <v>561000</v>
+        <v>269280</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C28" s="22" t="n">
-        <f aca="false">INDEX(Parameter!$E$25:$E$33,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
+        <f aca="false">INDEX(Parameter!$E$26:$E$34,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
         <v>0.1</v>
       </c>
       <c r="D28" s="26" t="n">
         <f aca="false">$D$16*C28</f>
-        <v>990000000</v>
+        <v>475200000</v>
       </c>
       <c r="E28" s="20" t="n">
         <f aca="false">IF($C$7&gt;0,D28/$C$7,0)</f>
-        <v>330000</v>
+        <v>158400</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C29" s="22" t="n">
-        <f aca="false">INDEX(Parameter!$F$25:$F$33,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
+        <f aca="false">INDEX(Parameter!$F$26:$F$34,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
         <v>0.09</v>
       </c>
       <c r="D29" s="26" t="n">
         <f aca="false">$D$16*C29</f>
-        <v>891000000</v>
+        <v>427680000</v>
       </c>
       <c r="E29" s="20" t="n">
         <f aca="false">IF($C$7&gt;0,D29/$C$7,0)</f>
-        <v>297000</v>
+        <v>142560</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C30" s="22" t="n">
-        <f aca="false">INDEX(Parameter!$G$25:$G$33,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
+        <f aca="false">INDEX(Parameter!$G$26:$G$34,MATCH($C$6,Parameter!$A$6:$A$14,0))</f>
         <v>0.07</v>
       </c>
       <c r="D30" s="26" t="n">
         <f aca="false">$D$16*C30</f>
-        <v>693000000</v>
+        <v>332640000</v>
       </c>
       <c r="E30" s="20" t="n">
         <f aca="false">IF($C$7&gt;0,D30/$C$7,0)</f>
-        <v>231000</v>
+        <v>110880</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C31" s="27" t="n">
         <f aca="false">SUM(C25:C30)</f>
@@ -1473,16 +1496,16 @@
       </c>
       <c r="D31" s="28" t="n">
         <f aca="false">SUM(D25:D30)</f>
-        <v>9900000000</v>
+        <v>4752000000</v>
       </c>
       <c r="E31" s="28" t="n">
         <f aca="false">SUM(E25:E30)</f>
-        <v>3300000</v>
+        <v>1584000</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="29" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C33" s="29"/>
       <c r="D33" s="29"/>
@@ -1520,7 +1543,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" error="Pilih dari daftar." errorStyle="stop" errorTitle="Pilihan tidak valid" operator="between" prompt="Mall atau Ruko" promptTitle="Pilih" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C9" type="list">
-      <formula1>Parameter!$A$19:$A$20</formula1>
+      <formula1>Parameter!$A$20:$A$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" error="Isi angka lebih dari 0." errorStyle="stop" errorTitle="Angka tidak valid" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C7:C8" type="decimal">
@@ -1544,7 +1567,7 @@
     <tabColor rgb="FFBF8F00"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -1555,12 +1578,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="30" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -1574,29 +1597,29 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5" s="32" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E5" s="32" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B6" s="33" t="n">
         <v>0.18</v>
@@ -1613,7 +1636,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B7" s="33" t="n">
         <v>0.2</v>
@@ -1630,7 +1653,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B8" s="33" t="n">
         <v>0.2</v>
@@ -1647,7 +1670,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B9" s="33" t="n">
         <v>0.2</v>
@@ -1664,7 +1687,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B10" s="33" t="n">
         <v>0.1</v>
@@ -1673,15 +1696,15 @@
         <v>0.16</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>2500000</v>
+        <v>800000</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>5000000</v>
+        <v>1300000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" s="33" t="n">
         <v>0.09</v>
@@ -1690,15 +1713,15 @@
         <v>0.13</v>
       </c>
       <c r="D11" s="18" t="n">
-        <v>2000000</v>
+        <v>1000000</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>4000000</v>
+        <v>1600000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B12" s="33" t="n">
         <v>0.04</v>
@@ -1715,7 +1738,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B13" s="33" t="n">
         <v>0.04</v>
@@ -1732,7 +1755,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B14" s="33" t="n">
         <v>0.04</v>
@@ -1749,122 +1772,99 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="31" t="s">
         <v>91</v>
       </c>
     </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="34" t="s">
+        <v>92</v>
+      </c>
+    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="34" t="s">
-        <v>92</v>
+      <c r="A18" s="31" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>93</v>
+      <c r="B19" s="35" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B20" s="35" t="n">
-        <v>0.85</v>
+        <v>43</v>
+      </c>
+      <c r="B20" s="36" t="n">
+        <v>1</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="31" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="B24" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24" s="32" t="s">
+      <c r="B21" s="36" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="31" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="D24" s="32" t="s">
+      <c r="C25" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="E24" s="32" t="s">
+      <c r="D25" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="F24" s="32" t="s">
+      <c r="E25" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="G24" s="32" t="s">
+      <c r="F25" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="21" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="str">
+      <c r="G25" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="H25" s="21" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="19" t="str">
         <f aca="false">A6</f>
         <v>Kafe / resto (F&amp;B)</v>
       </c>
-      <c r="B25" s="33" t="n">
+      <c r="B26" s="33" t="n">
         <v>0.25</v>
       </c>
-      <c r="C25" s="33" t="n">
+      <c r="C26" s="33" t="n">
         <v>0.15</v>
       </c>
-      <c r="D25" s="33" t="n">
+      <c r="D26" s="33" t="n">
         <v>0.3</v>
-      </c>
-      <c r="E25" s="33" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F25" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G25" s="33" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="H25" s="22" t="n">
-        <f aca="false">SUM(B25:G25)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="str">
-        <f aca="false">A7</f>
-        <v>Fashion / aksesoris</v>
-      </c>
-      <c r="B26" s="33" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C26" s="33" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="D26" s="33" t="n">
-        <v>0.25</v>
       </c>
       <c r="E26" s="33" t="n">
         <v>0.12</v>
       </c>
       <c r="F26" s="33" t="n">
-        <v>0.07</v>
+        <v>0.1</v>
       </c>
       <c r="G26" s="33" t="n">
         <v>0.08</v>
@@ -1876,23 +1876,23 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="str">
-        <f aca="false">A8</f>
-        <v>Salon</v>
+        <f aca="false">A7</f>
+        <v>Fashion / aksesoris</v>
       </c>
       <c r="B27" s="33" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C27" s="33" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D27" s="33" t="n">
         <v>0.25</v>
       </c>
-      <c r="C27" s="33" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D27" s="33" t="n">
-        <v>0.3</v>
-      </c>
       <c r="E27" s="33" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="F27" s="33" t="n">
-        <v>0.12</v>
+        <v>0.07</v>
       </c>
       <c r="G27" s="33" t="n">
         <v>0.08</v>
@@ -1904,11 +1904,11 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="str">
-        <f aca="false">A9</f>
-        <v>Klinik kecantikan / kesehatan</v>
+        <f aca="false">A8</f>
+        <v>Salon</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="C28" s="33" t="n">
         <v>0.15</v>
@@ -1920,7 +1920,7 @@
         <v>0.1</v>
       </c>
       <c r="F28" s="33" t="n">
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="G28" s="33" t="n">
         <v>0.08</v>
@@ -1932,23 +1932,23 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="str">
-        <f aca="false">A10</f>
-        <v>Furnitur &amp; dekorasi rumah (big-box)</v>
+        <f aca="false">A9</f>
+        <v>Klinik kecantikan / kesehatan</v>
       </c>
       <c r="B29" s="33" t="n">
-        <v>0.32</v>
+        <v>0.2</v>
       </c>
       <c r="C29" s="33" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="D29" s="33" t="n">
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="E29" s="33" t="n">
         <v>0.1</v>
       </c>
       <c r="F29" s="33" t="n">
-        <v>0.08</v>
+        <v>0.17</v>
       </c>
       <c r="G29" s="33" t="n">
         <v>0.08</v>
@@ -1960,26 +1960,26 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="str">
-        <f aca="false">A11</f>
-        <v>Perlengkapan rumah &amp; perkakas (big-box)</v>
+        <f aca="false">A10</f>
+        <v>Furnitur &amp; dekorasi rumah (big-box)</v>
       </c>
       <c r="B30" s="33" t="n">
-        <v>0.4</v>
+        <v>0.32</v>
       </c>
       <c r="C30" s="33" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="D30" s="33" t="n">
-        <v>0.17</v>
+        <v>0.24</v>
       </c>
       <c r="E30" s="33" t="n">
         <v>0.1</v>
       </c>
       <c r="F30" s="33" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="G30" s="33" t="n">
-        <v>0.07</v>
+        <v>0.08</v>
       </c>
       <c r="H30" s="22" t="n">
         <f aca="false">SUM(B30:G30)</f>
@@ -1988,26 +1988,26 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="str">
-        <f aca="false">A12</f>
-        <v>Apotek / toko kesehatan</v>
+        <f aca="false">A11</f>
+        <v>Perlengkapan rumah &amp; perkakas (big-box)</v>
       </c>
       <c r="B31" s="33" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="C31" s="33" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="D31" s="33" t="n">
-        <v>0.25</v>
+        <v>0.17</v>
       </c>
       <c r="E31" s="33" t="n">
         <v>0.1</v>
       </c>
       <c r="F31" s="33" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="G31" s="33" t="n">
         <v>0.07</v>
-      </c>
-      <c r="G31" s="33" t="n">
-        <v>0.08</v>
       </c>
       <c r="H31" s="22" t="n">
         <f aca="false">SUM(B31:G31)</f>
@@ -2016,17 +2016,17 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="str">
-        <f aca="false">A13</f>
-        <v>Minimarket / grocery</v>
+        <f aca="false">A12</f>
+        <v>Apotek / toko kesehatan</v>
       </c>
       <c r="B32" s="33" t="n">
         <v>0.35</v>
       </c>
       <c r="C32" s="33" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="D32" s="33" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="E32" s="33" t="n">
         <v>0.1</v>
@@ -2044,29 +2044,57 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="str">
+        <f aca="false">A13</f>
+        <v>Minimarket / grocery</v>
+      </c>
+      <c r="B33" s="33" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C33" s="33" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D33" s="33" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E33" s="33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F33" s="33" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="G33" s="33" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H33" s="22" t="n">
+        <f aca="false">SUM(B33:G33)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="19" t="str">
         <f aca="false">A14</f>
         <v>Elektronik / gadget</v>
       </c>
-      <c r="B33" s="33" t="n">
+      <c r="B34" s="33" t="n">
         <v>0.3</v>
       </c>
-      <c r="C33" s="33" t="n">
+      <c r="C34" s="33" t="n">
         <v>0.18</v>
       </c>
-      <c r="D33" s="33" t="n">
+      <c r="D34" s="33" t="n">
         <v>0.22</v>
       </c>
-      <c r="E33" s="33" t="n">
+      <c r="E34" s="33" t="n">
         <v>0.12</v>
       </c>
-      <c r="F33" s="33" t="n">
+      <c r="F34" s="33" t="n">
         <v>0.1</v>
       </c>
-      <c r="G33" s="33" t="n">
+      <c r="G34" s="33" t="n">
         <v>0.08</v>
       </c>
-      <c r="H33" s="22" t="n">
-        <f aca="false">SUM(B33:G33)</f>
+      <c r="H34" s="22" t="n">
+        <f aca="false">SUM(B34:G34)</f>
         <v>1</v>
       </c>
     </row>
@@ -2074,9 +2102,9 @@
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H25:H33">
+  <conditionalFormatting sqref="H26:H34">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
-      <formula>ROUND(H25,4)&lt;&gt;1</formula>
+      <formula>ROUND(H26,4)&lt;&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>